<commit_message>
- put aiengine as an option (selection field) - anonymize data of test & template
</commit_message>
<xml_diff>
--- a/partner_import_helper/data/Import Clients, Fournisseurs, Contacts (res.partner).xlsx
+++ b/partner_import_helper/data/Import Clients, Fournisseurs, Contacts (res.partner).xlsx
@@ -5,7 +5,7 @@
   <workbookPr backupFile="false" showObjects="all" date1904="false"/>
   <workbookProtection/>
   <bookViews>
-    <workbookView showHorizontalScroll="true" showVerticalScroll="true" showSheetTabs="true" xWindow="0" yWindow="0" windowWidth="16384" windowHeight="8192" tabRatio="500" firstSheet="0" activeTab="2"/>
+    <workbookView showHorizontalScroll="true" showVerticalScroll="true" showSheetTabs="true" xWindow="0" yWindow="0" windowWidth="16384" windowHeight="8192" tabRatio="500" firstSheet="0" activeTab="0"/>
   </bookViews>
   <sheets>
     <sheet name="companies" sheetId="1" state="visible" r:id="rId3"/>
@@ -23,7 +23,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="307" uniqueCount="134">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="307" uniqueCount="138">
   <si>
     <t xml:space="preserve">IDENTIFICATION</t>
   </si>
@@ -247,31 +247,31 @@
     <t xml:space="preserve">FRN001</t>
   </si>
   <si>
-    <t xml:space="preserve">ALUVAL</t>
-  </si>
-  <si>
-    <t xml:space="preserve">FR52948140546</t>
+    <t xml:space="preserve">Ma Société</t>
+  </si>
+  <si>
+    <t xml:space="preserve">FR00000000000</t>
   </si>
   <si>
     <t xml:space="preserve">'FR' ou 'Grande Bretagne'</t>
   </si>
   <si>
-    <t xml:space="preserve">10 rue perriere LA MEMBROLLE SUR LONGUENEE</t>
-  </si>
-  <si>
-    <t xml:space="preserve">LONGUENEE EN ANJOU</t>
-  </si>
-  <si>
-    <t xml:space="preserve">+34 2 40 78 77 32</t>
-  </si>
-  <si>
-    <t xml:space="preserve">06 68 49 89 60</t>
-  </si>
-  <si>
-    <t xml:space="preserve">arnaud.layec@akretion.com</t>
-  </si>
-  <si>
-    <t xml:space="preserve">https://www.akretion.com</t>
+    <t xml:space="preserve">10 rue de la cité</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Ma Ville</t>
+  </si>
+  <si>
+    <t xml:space="preserve">02 40 01 01 01</t>
+  </si>
+  <si>
+    <t xml:space="preserve">06 01 01 01 01</t>
+  </si>
+  <si>
+    <t xml:space="preserve">prenom.nom@email.com</t>
+  </si>
+  <si>
+    <t xml:space="preserve">https://www.company.com</t>
   </si>
   <si>
     <t xml:space="preserve">Banque &amp; Assurance, Transports, Energies, …</t>
@@ -283,28 +283,37 @@
     <t xml:space="preserve"> Bâtiment,Energie</t>
   </si>
   <si>
-    <t xml:space="preserve">Paul MICHEL</t>
+    <t xml:space="preserve">Prénom NOM</t>
   </si>
   <si>
     <t xml:space="preserve">Monsieur</t>
   </si>
   <si>
-    <t xml:space="preserve">3 allée des violettes</t>
-  </si>
-  <si>
-    <t xml:space="preserve">La Chapelle sur Erdre</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Julie LEBRUN</t>
+    <t xml:space="preserve">3 rue de la cité</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Mon Village</t>
+  </si>
+  <si>
+    <t xml:space="preserve">02 40 02 02 02</t>
+  </si>
+  <si>
+    <t xml:space="preserve">06 02 02 02 02</t>
   </si>
   <si>
     <t xml:space="preserve">Madame</t>
   </si>
   <si>
-    <t xml:space="preserve">12 chemin des embruns</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Paris</t>
+    <t xml:space="preserve">12 rue de la cité</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Ville3</t>
+  </si>
+  <si>
+    <t xml:space="preserve">02 40 03 03 03</t>
+  </si>
+  <si>
+    <t xml:space="preserve">06 03 03 03 03</t>
   </si>
   <si>
     <t xml:space="preserve">AUTRES CONTACTS</t>
@@ -322,7 +331,10 @@
     <t xml:space="preserve">contact</t>
   </si>
   <si>
-    <t xml:space="preserve">Directrice adjointe</t>
+    <t xml:space="preserve">Directrice</t>
+  </si>
+  <si>
+    <t xml:space="preserve">06 05 05 05 05</t>
   </si>
   <si>
     <t xml:space="preserve">Energie</t>
@@ -1491,7 +1503,7 @@
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="5" min="5" style="1" width="16.63"/>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="6" min="6" style="1" width="17.8"/>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="7" min="7" style="1" width="25.8"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="8" min="8" style="1" width="43.98"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="8" min="8" style="1" width="17.28"/>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="9" min="9" style="1" width="19.73"/>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="10" min="10" style="1" width="21.53"/>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="11" min="11" style="1" width="10.95"/>
@@ -1518,11 +1530,12 @@
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="33" min="33" style="1" width="17.92"/>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="34" min="34" style="1" width="22.44"/>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="35" min="35" style="1" width="15.6"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="36" min="36" style="1" width="12.5"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="36" min="36" style="1" width="13.53"/>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="37" min="37" style="1" width="11.86"/>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="38" min="38" style="1" width="16.37"/>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="39" min="39" style="1" width="15.47"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="41" min="40" style="1" width="13.15"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="40" min="40" style="1" width="22.95"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="41" min="41" style="1" width="13.15"/>
     <col collapsed="false" customWidth="false" hidden="false" outlineLevel="0" max="16374" min="42" style="1" width="10.16"/>
     <col collapsed="false" customWidth="false" hidden="false" outlineLevel="0" max="16384" min="16380" style="2" width="10.16"/>
   </cols>
@@ -1584,7 +1597,7 @@
       <c r="XEV1" s="2"/>
       <c r="XEW1" s="2"/>
       <c r="XEX1" s="2"/>
-      <c r="XEY1" s="0"/>
+      <c r="XEY1" s="2"/>
       <c r="XEZ1" s="2"/>
       <c r="XFA1" s="2"/>
       <c r="XFB1" s="2"/>
@@ -1679,7 +1692,7 @@
       <c r="XEV2" s="16"/>
       <c r="XEW2" s="16"/>
       <c r="XEX2" s="2"/>
-      <c r="XEY2" s="0"/>
+      <c r="XEY2" s="2"/>
       <c r="XEZ2" s="2"/>
       <c r="XFA2" s="2"/>
       <c r="XFB2" s="2"/>
@@ -1814,7 +1827,7 @@
       <c r="XEV3" s="2"/>
       <c r="XEW3" s="2"/>
       <c r="XEX3" s="2"/>
-      <c r="XEY3" s="0"/>
+      <c r="XEY3" s="2"/>
       <c r="XEZ3" s="2"/>
       <c r="XFA3" s="2"/>
       <c r="XFB3" s="2"/>
@@ -1963,7 +1976,7 @@
         <v>75</v>
       </c>
       <c r="F5" s="1" t="n">
-        <v>44316952400120</v>
+        <v>0</v>
       </c>
       <c r="G5" s="1" t="s">
         <v>76</v>
@@ -1975,7 +1988,7 @@
         <v>78</v>
       </c>
       <c r="K5" s="1" t="n">
-        <v>49770</v>
+        <v>11111</v>
       </c>
       <c r="L5" s="12" t="s">
         <v>79</v>
@@ -2011,13 +2024,13 @@
         <v>89</v>
       </c>
       <c r="AA5" s="1" t="n">
-        <v>44240</v>
+        <v>12333</v>
       </c>
       <c r="AB5" s="12" t="s">
-        <v>79</v>
+        <v>90</v>
       </c>
       <c r="AC5" s="12" t="s">
-        <v>80</v>
+        <v>91</v>
       </c>
       <c r="AD5" s="21" t="s">
         <v>81</v>
@@ -2026,25 +2039,25 @@
         <v>84</v>
       </c>
       <c r="AF5" s="1" t="s">
-        <v>90</v>
+        <v>86</v>
       </c>
       <c r="AG5" s="1" t="s">
-        <v>91</v>
+        <v>92</v>
       </c>
       <c r="AH5" s="1" t="s">
-        <v>92</v>
+        <v>93</v>
       </c>
       <c r="AJ5" s="1" t="s">
-        <v>93</v>
+        <v>94</v>
       </c>
       <c r="AK5" s="1" t="n">
-        <v>75018</v>
+        <v>15000</v>
       </c>
       <c r="AL5" s="12" t="s">
-        <v>79</v>
+        <v>95</v>
       </c>
       <c r="AM5" s="12" t="s">
-        <v>80</v>
+        <v>96</v>
       </c>
       <c r="AN5" s="21" t="s">
         <v>81</v>
@@ -2058,10 +2071,9 @@
     <mergeCell ref="B1:F1"/>
   </mergeCells>
   <hyperlinks>
-    <hyperlink ref="N5" r:id="rId1" display="arnaud.layec@akretion.com"/>
-    <hyperlink ref="O5" r:id="rId2" display="https://www.akretion.com"/>
-    <hyperlink ref="AD5" r:id="rId3" display="arnaud.layec@akretion.com"/>
-    <hyperlink ref="AN5" r:id="rId4" display="arnaud.layec@akretion.com"/>
+    <hyperlink ref="N5" r:id="rId1" display="prenom.nom@email.com"/>
+    <hyperlink ref="O5" r:id="rId2" display="https://www.company.com"/>
+    <hyperlink ref="AN5" r:id="rId3" display="prenom.nom@email.com"/>
   </hyperlinks>
   <printOptions headings="false" gridLines="false" gridLinesSet="true" horizontalCentered="false" verticalCentered="false"/>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.511811023622047" footer="0.511811023622047"/>
@@ -2091,12 +2103,13 @@
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="10" min="10" style="2" width="11.47"/>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="11" min="11" style="2" width="16.37"/>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="12" min="12" style="2" width="15.09"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="14" min="13" style="2" width="12.76"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="13" min="13" style="2" width="22.95"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="14" min="14" style="2" width="12.76"/>
   </cols>
   <sheetData>
     <row r="1" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A1" s="22" t="s">
-        <v>94</v>
+        <v>97</v>
       </c>
       <c r="B1" s="22"/>
       <c r="C1" s="22"/>
@@ -2168,16 +2181,16 @@
         <v>32</v>
       </c>
       <c r="C3" s="20" t="s">
-        <v>95</v>
+        <v>98</v>
       </c>
       <c r="D3" s="20" t="s">
         <v>33</v>
       </c>
       <c r="E3" s="20" t="s">
-        <v>96</v>
+        <v>99</v>
       </c>
       <c r="F3" s="20" t="s">
-        <v>97</v>
+        <v>100</v>
       </c>
       <c r="G3" s="20" t="s">
         <v>37</v>
@@ -2215,32 +2228,32 @@
         <v>73</v>
       </c>
       <c r="C4" s="1" t="s">
-        <v>98</v>
+        <v>101</v>
       </c>
       <c r="D4" s="1" t="s">
-        <v>90</v>
+        <v>86</v>
       </c>
       <c r="E4" s="1" t="s">
-        <v>91</v>
+        <v>92</v>
       </c>
       <c r="F4" s="1" t="s">
-        <v>99</v>
+        <v>102</v>
       </c>
       <c r="G4" s="1" t="s">
-        <v>92</v>
+        <v>88</v>
       </c>
       <c r="H4" s="1"/>
       <c r="I4" s="1" t="s">
-        <v>93</v>
+        <v>15</v>
       </c>
       <c r="J4" s="1" t="n">
-        <v>75018</v>
+        <v>15000</v>
       </c>
       <c r="K4" s="12" t="s">
         <v>79</v>
       </c>
       <c r="L4" s="12" t="s">
-        <v>80</v>
+        <v>103</v>
       </c>
       <c r="M4" s="12" t="s">
         <v>81</v>
@@ -2249,12 +2262,12 @@
         <v>84</v>
       </c>
       <c r="O4" s="1" t="s">
-        <v>100</v>
+        <v>104</v>
       </c>
     </row>
   </sheetData>
   <hyperlinks>
-    <hyperlink ref="M4" r:id="rId1" display="arnaud.layec@akretion.com"/>
+    <hyperlink ref="M4" r:id="rId1" display="prenom.nom@email.com"/>
   </hyperlinks>
   <printOptions headings="false" gridLines="false" gridLinesSet="true" horizontalCentered="false" verticalCentered="false"/>
   <pageMargins left="0.7875" right="0.7875" top="1.05277777777778" bottom="1.05277777777778" header="0.7875" footer="0.7875"/>
@@ -2277,8 +2290,7 @@
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="2" width="21.69"/>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="2" min="2" style="2" width="20.76"/>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="3" min="3" style="2" width="20.5"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="4" min="4" style="2" width="16.94"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="5" min="5" style="0" width="16.94"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="5" min="4" style="2" width="16.94"/>
   </cols>
   <sheetData>
     <row r="1" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -2286,7 +2298,7 @@
         <v>7</v>
       </c>
       <c r="B1" s="7" t="s">
-        <v>101</v>
+        <v>105</v>
       </c>
       <c r="C1" s="7" t="s">
         <v>21</v>
@@ -2339,7 +2351,6 @@
       <c r="B4" s="1" t="s">
         <v>73</v>
       </c>
-      <c r="E4" s="2"/>
     </row>
   </sheetData>
   <printOptions headings="false" gridLines="false" gridLinesSet="true" horizontalCentered="false" verticalCentered="false"/>
@@ -2367,15 +2378,15 @@
   <sheetData>
     <row r="1" customFormat="false" ht="26.7" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A1" s="26" t="s">
-        <v>102</v>
+        <v>106</v>
       </c>
       <c r="B1" s="26" t="s">
-        <v>103</v>
+        <v>107</v>
       </c>
     </row>
     <row r="2" customFormat="false" ht="195.6" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A2" s="27" t="s">
-        <v>104</v>
+        <v>108</v>
       </c>
       <c r="B2" s="27"/>
     </row>
@@ -2389,10 +2400,10 @@
     </row>
     <row r="5" s="2" customFormat="true" ht="16.4" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A5" s="29" t="s">
-        <v>103</v>
+        <v>107</v>
       </c>
       <c r="B5" s="30" t="s">
-        <v>105</v>
+        <v>109</v>
       </c>
       <c r="D5" s="25"/>
     </row>
@@ -2408,7 +2419,7 @@
         <v>31</v>
       </c>
       <c r="B7" s="24" t="s">
-        <v>106</v>
+        <v>110</v>
       </c>
     </row>
     <row r="8" customFormat="false" ht="31.3" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -2416,7 +2427,7 @@
         <v>32</v>
       </c>
       <c r="B8" s="24" t="s">
-        <v>107</v>
+        <v>111</v>
       </c>
       <c r="C8" s="2"/>
       <c r="D8" s="2"/>
@@ -2436,7 +2447,7 @@
         <v>34</v>
       </c>
       <c r="B10" s="24" t="s">
-        <v>108</v>
+        <v>112</v>
       </c>
       <c r="C10" s="2"/>
       <c r="D10" s="2"/>
@@ -2446,7 +2457,7 @@
         <v>35</v>
       </c>
       <c r="B11" s="24" t="s">
-        <v>109</v>
+        <v>113</v>
       </c>
       <c r="C11" s="2"/>
     </row>
@@ -2462,7 +2473,7 @@
         <v>36</v>
       </c>
       <c r="B13" s="24" t="s">
-        <v>110</v>
+        <v>114</v>
       </c>
     </row>
     <row r="14" customFormat="false" ht="16.4" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -2470,7 +2481,7 @@
         <v>37</v>
       </c>
       <c r="B14" s="24" t="s">
-        <v>111</v>
+        <v>115</v>
       </c>
     </row>
     <row r="15" customFormat="false" ht="16.4" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -2478,7 +2489,7 @@
         <v>38</v>
       </c>
       <c r="B15" s="24" t="s">
-        <v>111</v>
+        <v>115</v>
       </c>
     </row>
     <row r="16" customFormat="false" ht="16.4" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -2486,7 +2497,7 @@
         <v>39</v>
       </c>
       <c r="B16" s="24" t="s">
-        <v>111</v>
+        <v>115</v>
       </c>
     </row>
     <row r="17" customFormat="false" ht="16.4" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -2494,7 +2505,7 @@
         <v>40</v>
       </c>
       <c r="B17" s="24" t="s">
-        <v>112</v>
+        <v>116</v>
       </c>
     </row>
     <row r="18" customFormat="false" ht="31.3" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -2502,7 +2513,7 @@
         <v>41</v>
       </c>
       <c r="B18" s="24" t="s">
-        <v>113</v>
+        <v>117</v>
       </c>
     </row>
     <row r="19" customFormat="false" ht="16.4" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -2510,7 +2521,7 @@
         <v>42</v>
       </c>
       <c r="B19" s="24" t="s">
-        <v>114</v>
+        <v>118</v>
       </c>
     </row>
     <row r="20" customFormat="false" ht="16.4" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -2518,7 +2529,7 @@
         <v>43</v>
       </c>
       <c r="B20" s="24" t="s">
-        <v>115</v>
+        <v>119</v>
       </c>
     </row>
     <row r="21" customFormat="false" ht="16.4" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -2526,7 +2537,7 @@
         <v>44</v>
       </c>
       <c r="B21" s="24" t="s">
-        <v>111</v>
+        <v>115</v>
       </c>
     </row>
     <row r="22" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -2540,7 +2551,7 @@
         <v>45</v>
       </c>
       <c r="B23" s="24" t="s">
-        <v>116</v>
+        <v>120</v>
       </c>
     </row>
     <row r="24" customFormat="false" ht="46.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -2548,7 +2559,7 @@
         <v>46</v>
       </c>
       <c r="B24" s="24" t="s">
-        <v>117</v>
+        <v>121</v>
       </c>
     </row>
     <row r="25" customFormat="false" ht="16.4" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -2556,7 +2567,7 @@
         <v>47</v>
       </c>
       <c r="B25" s="24" t="s">
-        <v>118</v>
+        <v>122</v>
       </c>
     </row>
     <row r="26" customFormat="false" ht="31.3" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -2564,7 +2575,7 @@
         <v>48</v>
       </c>
       <c r="B26" s="24" t="s">
-        <v>119</v>
+        <v>123</v>
       </c>
     </row>
     <row r="27" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -2578,7 +2589,7 @@
         <v>49</v>
       </c>
       <c r="B28" s="36" t="s">
-        <v>120</v>
+        <v>124</v>
       </c>
     </row>
     <row r="29" customFormat="false" ht="61.15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -2586,7 +2597,7 @@
         <v>50</v>
       </c>
       <c r="B29" s="24" t="s">
-        <v>121</v>
+        <v>125</v>
       </c>
     </row>
     <row r="30" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -2600,7 +2611,7 @@
         <v>51</v>
       </c>
       <c r="B31" s="39" t="s">
-        <v>122</v>
+        <v>126</v>
       </c>
       <c r="D31" s="40"/>
     </row>
@@ -2609,7 +2620,7 @@
         <v>52</v>
       </c>
       <c r="B32" s="41" t="s">
-        <v>123</v>
+        <v>127</v>
       </c>
     </row>
     <row r="33" customFormat="false" ht="13.8" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -2617,7 +2628,7 @@
         <v>53</v>
       </c>
       <c r="B33" s="42" t="s">
-        <v>124</v>
+        <v>128</v>
       </c>
     </row>
     <row r="34" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -2673,7 +2684,7 @@
         <v>61</v>
       </c>
       <c r="B42" s="41" t="s">
-        <v>124</v>
+        <v>128</v>
       </c>
     </row>
     <row r="43" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -2732,7 +2743,7 @@
     </row>
     <row r="53" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A53" s="22" t="s">
-        <v>125</v>
+        <v>129</v>
       </c>
       <c r="B53" s="22"/>
     </row>
@@ -2741,7 +2752,7 @@
         <v>32</v>
       </c>
       <c r="B54" s="36" t="s">
-        <v>126</v>
+        <v>130</v>
       </c>
     </row>
     <row r="55" customFormat="false" ht="31.3" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -2749,15 +2760,15 @@
         <v>31</v>
       </c>
       <c r="B55" s="36" t="s">
-        <v>127</v>
+        <v>131</v>
       </c>
     </row>
     <row r="56" customFormat="false" ht="120.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A56" s="38" t="s">
-        <v>95</v>
+        <v>98</v>
       </c>
       <c r="B56" s="44" t="s">
-        <v>128</v>
+        <v>132</v>
       </c>
     </row>
     <row r="57" customFormat="false" ht="13.8" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -2765,21 +2776,21 @@
         <v>33</v>
       </c>
       <c r="B57" s="42" t="s">
-        <v>129</v>
+        <v>133</v>
       </c>
     </row>
     <row r="58" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A58" s="38" t="s">
-        <v>96</v>
+        <v>99</v>
       </c>
       <c r="B58" s="42"/>
     </row>
     <row r="59" customFormat="false" ht="16.4" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A59" s="38" t="s">
-        <v>97</v>
+        <v>100</v>
       </c>
       <c r="B59" s="36" t="s">
-        <v>130</v>
+        <v>134</v>
       </c>
     </row>
     <row r="60" customFormat="false" ht="13.8" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -2787,7 +2798,7 @@
         <v>37</v>
       </c>
       <c r="B60" s="42" t="s">
-        <v>129</v>
+        <v>133</v>
       </c>
     </row>
     <row r="61" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -2801,7 +2812,7 @@
         <v>39</v>
       </c>
       <c r="B62" s="42" t="s">
-        <v>129</v>
+        <v>133</v>
       </c>
     </row>
     <row r="63" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -2815,7 +2826,7 @@
         <v>41</v>
       </c>
       <c r="B64" s="42" t="s">
-        <v>129</v>
+        <v>133</v>
       </c>
     </row>
     <row r="65" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -2835,12 +2846,12 @@
         <v>49</v>
       </c>
       <c r="B67" s="42" t="s">
-        <v>129</v>
+        <v>133</v>
       </c>
     </row>
     <row r="69" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A69" s="45" t="s">
-        <v>131</v>
+        <v>135</v>
       </c>
       <c r="B69" s="45"/>
     </row>
@@ -2849,7 +2860,7 @@
         <v>32</v>
       </c>
       <c r="B70" s="24" t="s">
-        <v>132</v>
+        <v>136</v>
       </c>
     </row>
     <row r="71" customFormat="false" ht="13.8" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -2857,7 +2868,7 @@
         <v>46</v>
       </c>
       <c r="B71" s="46" t="s">
-        <v>133</v>
+        <v>137</v>
       </c>
     </row>
     <row r="72" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">

</xml_diff>